<commit_message>
feat: bulk 005 done
</commit_message>
<xml_diff>
--- a/fixtures/student-data-alright - verifyID.xlsx
+++ b/fixtures/student-data-alright - verifyID.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marango\Desktop\suite Pae\fixtures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marango\Desktop\Pae-Suite\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A802D7-97F2-42B9-B910-7A5DFB7E69C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35055" yWindow="2040" windowWidth="22665" windowHeight="6960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>